<commit_message>
Support the new temporal-only SSL strategy.
</commit_message>
<xml_diff>
--- a/notebooks/Multi-View Model Performance.xlsx
+++ b/notebooks/Multi-View Model Performance.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28926"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28928"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBDCECDB-A5B6-4C30-A980-59E68B4EB0E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uflorida-my.sharepoint.com/personal/cli2_ufl_edu/Documents/Students/DanielPetti/Projects/SSL/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1B969B0-5D00-43E5-9700-BA271903AEF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MoCo 2-View" sheetId="1" r:id="rId1"/>
@@ -97,7 +102,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,6 +123,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7.5"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -141,10 +154,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -580,10 +603,10 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C5">
         <v>0.76500439027886902</v>
@@ -603,10 +626,10 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C6">
         <v>0.76180922172575305</v>
@@ -626,10 +649,10 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C7">
         <v>0.76253275192831904</v>
@@ -718,10 +741,10 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C11">
         <v>0.76755459472681598</v>
@@ -741,10 +764,10 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C12">
         <v>0.76825623988879599</v>
@@ -764,10 +787,10 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C13">
         <v>0.76916787618520699</v>
@@ -856,10 +879,10 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17">
         <v>0.77702683447157805</v>
@@ -879,10 +902,10 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C18">
         <v>0.778742528240427</v>
@@ -902,10 +925,10 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19">
         <v>0.78018891196329099</v>
@@ -994,10 +1017,10 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C23">
         <v>0.75318327207256397</v>
@@ -1017,10 +1040,10 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B24">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C24">
         <v>0.75198592725812996</v>
@@ -1040,10 +1063,10 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B25">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C25">
         <v>0.74620133087598095</v>
@@ -1063,10 +1086,10 @@
     </row>
     <row r="26" spans="1:7">
       <c r="A26">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B26">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C26">
         <v>0.72817057144126296</v>
@@ -1086,10 +1109,10 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B27">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C27">
         <v>0.72762707620522604</v>
@@ -1109,10 +1132,10 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B28">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C28">
         <v>0.72445222219501004</v>
@@ -1201,10 +1224,10 @@
     </row>
     <row r="32" spans="1:7">
       <c r="A32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B32">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C32">
         <v>0.677680801257739</v>
@@ -1224,10 +1247,10 @@
     </row>
     <row r="33" spans="1:7">
       <c r="A33">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B33">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C33">
         <v>0.673136032211752</v>
@@ -1247,10 +1270,10 @@
     </row>
     <row r="34" spans="1:7">
       <c r="A34">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B34">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C34">
         <v>0.69429659170329505</v>
@@ -1338,11 +1361,11 @@
       </c>
     </row>
     <row r="38" spans="1:7">
-      <c r="A38">
-        <v>3</v>
+      <c r="A38" s="6">
+        <v>4</v>
       </c>
       <c r="B38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C38">
         <v>0.75895655532336304</v>
@@ -1362,10 +1385,10 @@
     </row>
     <row r="39" spans="1:7">
       <c r="A39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B39">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C39">
         <v>0.76363757878805405</v>
@@ -1385,10 +1408,10 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B40">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C40">
         <v>0.74716368383426801</v>
@@ -1408,10 +1431,10 @@
     </row>
     <row r="41" spans="1:7">
       <c r="A41">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B41">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C41">
         <v>0.68953715034666296</v>
@@ -1431,10 +1454,10 @@
     </row>
     <row r="42" spans="1:7">
       <c r="A42">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B42">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C42">
         <v>0.70695436180968196</v>
@@ -1454,10 +1477,10 @@
     </row>
     <row r="43" spans="1:7">
       <c r="A43">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B43">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C43">
         <v>0.72149668499285302</v>
@@ -1578,11 +1601,11 @@
       <c r="B2">
         <v>5</v>
       </c>
-      <c r="C2">
-        <v>0.59305595052890103</v>
-      </c>
-      <c r="D2">
-        <v>0.27343305258717898</v>
+      <c r="C2" s="3">
+        <v>0.59300632198973002</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0.27374453159859802</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1592,11 +1615,11 @@
       <c r="B3">
         <v>5</v>
       </c>
-      <c r="C3">
-        <v>0.58384183851145499</v>
-      </c>
-      <c r="D3">
-        <v>0.27061598327283998</v>
+      <c r="C3" s="3">
+        <v>0.60405341847307503</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.27394701669018201</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1606,11 +1629,11 @@
       <c r="B4">
         <v>5</v>
       </c>
-      <c r="C4">
-        <v>0.598127399477837</v>
-      </c>
-      <c r="D4">
-        <v>0.27357281642356102</v>
+      <c r="C4" s="3">
+        <v>0.58663858773467203</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0.26676071413371599</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1620,11 +1643,11 @@
       <c r="B5">
         <v>5</v>
       </c>
-      <c r="C5">
-        <v>0.66612746806866896</v>
-      </c>
-      <c r="D5">
-        <v>0.33431712671902702</v>
+      <c r="C5" s="3">
+        <v>0.63639784526003695</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.31303557077088501</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1634,11 +1657,11 @@
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6">
-        <v>0.67212229370109899</v>
-      </c>
-      <c r="D6">
-        <v>0.33701279089466701</v>
+      <c r="C6" s="3">
+        <v>0.65880126575534703</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0.32492050613675999</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1648,11 +1671,11 @@
       <c r="B7">
         <v>5</v>
       </c>
-      <c r="C7">
-        <v>0.67150823270761995</v>
-      </c>
-      <c r="D7">
-        <v>0.33274680436163301</v>
+      <c r="C7" s="3">
+        <v>0.64783348609976898</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0.31956848313914799</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1662,11 +1685,11 @@
       <c r="B8">
         <v>4</v>
       </c>
-      <c r="C8">
-        <v>0.69625045549318298</v>
-      </c>
-      <c r="D8">
-        <v>0.34764152805424697</v>
+      <c r="C8" s="3">
+        <v>0.60394666873477498</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.28025956029885901</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1676,11 +1699,11 @@
       <c r="B9">
         <v>4</v>
       </c>
-      <c r="C9">
-        <v>0.69617214667242</v>
-      </c>
-      <c r="D9">
-        <v>0.35006971367738499</v>
+      <c r="C9" s="3">
+        <v>0.593117247745229</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0.28032457624305401</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1690,11 +1713,11 @@
       <c r="B10">
         <v>4</v>
       </c>
-      <c r="C10">
-        <v>0.69290093209805004</v>
-      </c>
-      <c r="D10">
-        <v>0.34525474887567398</v>
+      <c r="C10" s="3">
+        <v>0.60913112949933401</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0.28567668099469501</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1704,11 +1727,11 @@
       <c r="B11">
         <v>5</v>
       </c>
-      <c r="C11">
-        <v>0.638997026556549</v>
-      </c>
-      <c r="D11">
-        <v>0.30474398127739799</v>
+      <c r="C11" s="3">
+        <v>0.656977915880958</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0.31419609438869101</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -1718,11 +1741,11 @@
       <c r="B12">
         <v>5</v>
       </c>
-      <c r="C12">
-        <v>0.63108994643798599</v>
-      </c>
-      <c r="D12">
-        <v>0.30631787402558902</v>
+      <c r="C12" s="3">
+        <v>0.64074770430127503</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0.31494074182973197</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -1732,11 +1755,11 @@
       <c r="B13">
         <v>5</v>
       </c>
-      <c r="C13">
-        <v>0.63086757291177697</v>
-      </c>
-      <c r="D13">
-        <v>0.30575853833898398</v>
+      <c r="C13" s="3">
+        <v>0.63649739049634402</v>
+      </c>
+      <c r="D13" s="5">
+        <v>0.31348085400884101</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -1746,11 +1769,11 @@
       <c r="B14">
         <v>4</v>
       </c>
-      <c r="C14">
-        <v>0.64047142831600501</v>
-      </c>
-      <c r="D14">
-        <v>0.31104307878981802</v>
+      <c r="C14" s="3">
+        <v>0.63632577205388596</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.30437135761418999</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1760,11 +1783,11 @@
       <c r="B15">
         <v>4</v>
       </c>
-      <c r="C15">
-        <v>0.64199924832201904</v>
-      </c>
-      <c r="D15">
-        <v>0.31132126433035101</v>
+      <c r="C15" s="3">
+        <v>0.63885091028904295</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.30644733200641999</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -1774,11 +1797,11 @@
       <c r="B16">
         <v>4</v>
       </c>
-      <c r="C16">
-        <v>0.64507782626102195</v>
-      </c>
-      <c r="D16">
-        <v>0.31219064993561002</v>
+      <c r="C16" s="3">
+        <v>0.64296240168534502</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0.30830246842466602</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1788,11 +1811,11 @@
       <c r="B17">
         <v>3</v>
       </c>
-      <c r="C17">
-        <v>0.48816504687328499</v>
-      </c>
-      <c r="D17">
-        <v>0.20008933780860999</v>
+      <c r="C17" s="3">
+        <v>0.70527301963742395</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.35167819280106699</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1802,11 +1825,11 @@
       <c r="B18">
         <v>3</v>
       </c>
-      <c r="C18">
-        <v>0.47255764099498498</v>
-      </c>
-      <c r="D18">
-        <v>0.189701995517327</v>
+      <c r="C18" s="3">
+        <v>0.70573799323816999</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.35397870881009202</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1816,11 +1839,11 @@
       <c r="B19">
         <v>3</v>
       </c>
-      <c r="C19">
-        <v>0.46914565911740103</v>
-      </c>
-      <c r="D19">
-        <v>0.18801841384621901</v>
+      <c r="C19" s="3">
+        <v>0.70518690876853896</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.353112386793418</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -1830,11 +1853,11 @@
       <c r="B20">
         <v>5</v>
       </c>
-      <c r="C20">
-        <v>0.67967297049342001</v>
-      </c>
-      <c r="D20">
-        <v>0.34111261653748098</v>
+      <c r="C20" s="3">
+        <v>0.66371957859686104</v>
+      </c>
+      <c r="D20" s="4">
+        <v>0.32847072054934001</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -1844,11 +1867,11 @@
       <c r="B21">
         <v>5</v>
       </c>
-      <c r="C21">
-        <v>0.66837027801300397</v>
-      </c>
-      <c r="D21">
-        <v>0.33064631979027598</v>
+      <c r="C21" s="3">
+        <v>0.66239912195740502</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0.325467965150469</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -1858,11 +1881,11 @@
       <c r="B22">
         <v>5</v>
       </c>
-      <c r="C22">
-        <v>0.67361141385202705</v>
-      </c>
-      <c r="D22">
-        <v>0.33388309292541801</v>
+      <c r="C22" s="3">
+        <v>0.66686208161716998</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0.32907092682217098</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -1872,11 +1895,11 @@
       <c r="B23">
         <v>4</v>
       </c>
-      <c r="C23">
-        <v>0.61850397884244601</v>
-      </c>
-      <c r="D23">
-        <v>0.308057876291849</v>
+      <c r="C23" s="3">
+        <v>0.662436975924237</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0.32923328831187598</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -1886,11 +1909,11 @@
       <c r="B24">
         <v>4</v>
       </c>
-      <c r="C24">
-        <v>0.64209289495295796</v>
-      </c>
-      <c r="D24">
-        <v>0.316561359431075</v>
+      <c r="C24" s="3">
+        <v>0.66937806162956404</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0.33197003282206899</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -1900,11 +1923,11 @@
       <c r="B25">
         <v>4</v>
       </c>
-      <c r="C25">
-        <v>0.62375455653050005</v>
-      </c>
-      <c r="D25">
-        <v>0.31252878544084101</v>
+      <c r="C25" s="3">
+        <v>0.66787870747063005</v>
+      </c>
+      <c r="D25" s="3">
+        <v>0.33309990514475302</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -1914,11 +1937,11 @@
       <c r="B26">
         <v>3</v>
       </c>
-      <c r="C26">
-        <v>0.69021250066669004</v>
-      </c>
-      <c r="D26">
-        <v>0.345062046724609</v>
+      <c r="C26" s="3">
+        <v>0.67494798831704195</v>
+      </c>
+      <c r="D26" s="3">
+        <v>0.33157265559993898</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -1928,11 +1951,11 @@
       <c r="B27">
         <v>3</v>
       </c>
-      <c r="C27">
-        <v>0.68544534398198498</v>
-      </c>
-      <c r="D27">
-        <v>0.34192979433891202</v>
+      <c r="C27" s="3">
+        <v>0.67170134253092195</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0.32843756250634298</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1942,11 +1965,11 @@
       <c r="B28">
         <v>3</v>
       </c>
-      <c r="C28">
-        <v>0.67460089150611102</v>
-      </c>
-      <c r="D28">
-        <v>0.347430623417264</v>
+      <c r="C28" s="3">
+        <v>0.66449688932374895</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0.32875553874810298</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -1956,11 +1979,11 @@
       <c r="B29">
         <v>2</v>
       </c>
-      <c r="C29">
-        <v>0.61102074670522599</v>
-      </c>
-      <c r="D29">
-        <v>0.28996447579707901</v>
+      <c r="C29" s="3">
+        <v>0.63659116702379204</v>
+      </c>
+      <c r="D29" s="3">
+        <v>0.31284158491745301</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -1970,11 +1993,11 @@
       <c r="B30">
         <v>2</v>
       </c>
-      <c r="C30">
-        <v>0.61589261142267704</v>
-      </c>
-      <c r="D30">
-        <v>0.290675444355812</v>
+      <c r="C30" s="3">
+        <v>0.65352407882072705</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0.31591850139724298</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -1984,11 +2007,11 @@
       <c r="B31">
         <v>2</v>
       </c>
-      <c r="C31">
-        <v>0.60872302746398899</v>
-      </c>
-      <c r="D31">
-        <v>0.28854691082343698</v>
+      <c r="C31" s="3">
+        <v>0.64962338197867997</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0.31363621451157803</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -1998,11 +2021,11 @@
       <c r="B32">
         <v>5</v>
       </c>
-      <c r="C32">
-        <v>0.55585232127376005</v>
-      </c>
-      <c r="D32">
-        <v>0.24776413489846</v>
+      <c r="C32" s="3">
+        <v>0.690143329623223</v>
+      </c>
+      <c r="D32" s="3">
+        <v>0.34981218454072499</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2012,11 +2035,11 @@
       <c r="B33">
         <v>5</v>
       </c>
-      <c r="C33">
-        <v>0.577844206656278</v>
-      </c>
-      <c r="D33">
-        <v>0.26362788286708799</v>
+      <c r="C33" s="3">
+        <v>0.68535538389313</v>
+      </c>
+      <c r="D33" s="3">
+        <v>0.34353076746273098</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2026,11 +2049,11 @@
       <c r="B34">
         <v>5</v>
       </c>
-      <c r="C34">
-        <v>0.57296775687735002</v>
-      </c>
-      <c r="D34">
-        <v>0.25935177276216398</v>
+      <c r="C34" s="3">
+        <v>0.69384862674761205</v>
+      </c>
+      <c r="D34" s="3">
+        <v>0.34890205169459598</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2040,11 +2063,11 @@
       <c r="B35">
         <v>1</v>
       </c>
-      <c r="C35">
-        <v>0.68088258723521899</v>
-      </c>
-      <c r="D35">
-        <v>0.33513671190496302</v>
+      <c r="C35" s="3">
+        <v>0.64309666777063701</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0.31436210810308002</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2054,11 +2077,11 @@
       <c r="B36">
         <v>1</v>
       </c>
-      <c r="C36">
-        <v>0.68118662577903799</v>
-      </c>
-      <c r="D36">
-        <v>0.335918165984402</v>
+      <c r="C36" s="3">
+        <v>0.63701599623587202</v>
+      </c>
+      <c r="D36" s="3">
+        <v>0.31580686040626998</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2068,11 +2091,11 @@
       <c r="B37">
         <v>1</v>
       </c>
-      <c r="C37">
-        <v>0.66757221467110195</v>
-      </c>
-      <c r="D37">
-        <v>0.33673522916325999</v>
+      <c r="C37" s="3">
+        <v>0.63965794156252398</v>
+      </c>
+      <c r="D37" s="3">
+        <v>0.31041297564123399</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2082,11 +2105,11 @@
       <c r="B38">
         <v>4</v>
       </c>
-      <c r="C38">
-        <v>0.58532945572664896</v>
-      </c>
-      <c r="D38">
-        <v>0.26882922438526202</v>
+      <c r="C38" s="3">
+        <v>0.64124200528294495</v>
+      </c>
+      <c r="D38" s="3">
+        <v>0.31605143933875901</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -2096,11 +2119,11 @@
       <c r="B39">
         <v>4</v>
       </c>
-      <c r="C39">
-        <v>0.57665307817762501</v>
-      </c>
-      <c r="D39">
-        <v>0.26350459748904698</v>
+      <c r="C39" s="3">
+        <v>0.64464054634439705</v>
+      </c>
+      <c r="D39" s="3">
+        <v>0.31708836480848601</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -2110,11 +2133,11 @@
       <c r="B40">
         <v>4</v>
       </c>
-      <c r="C40">
-        <v>0.57312169423263204</v>
-      </c>
-      <c r="D40">
-        <v>0.26346657283492703</v>
+      <c r="C40" s="3">
+        <v>0.63899149728593796</v>
+      </c>
+      <c r="D40" s="3">
+        <v>0.31247478332154999</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -2124,11 +2147,11 @@
       <c r="B41">
         <v>3</v>
       </c>
-      <c r="C41">
-        <v>0.653416493609841</v>
-      </c>
-      <c r="D41">
-        <v>0.33371720891706202</v>
+      <c r="C41" s="3">
+        <v>0.66988773247854605</v>
+      </c>
+      <c r="D41" s="3">
+        <v>0.34113238221706099</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -2138,11 +2161,11 @@
       <c r="B42">
         <v>3</v>
       </c>
-      <c r="C42">
-        <v>0.65153113319676903</v>
-      </c>
-      <c r="D42">
-        <v>0.33046189255458402</v>
+      <c r="C42" s="3">
+        <v>0.67295465836403301</v>
+      </c>
+      <c r="D42" s="3">
+        <v>0.34087884879851299</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -2152,11 +2175,11 @@
       <c r="B43">
         <v>3</v>
       </c>
-      <c r="C43">
-        <v>0.66773682802428402</v>
-      </c>
-      <c r="D43">
-        <v>0.33636085502820101</v>
+      <c r="C43" s="3">
+        <v>0.67245928204404504</v>
+      </c>
+      <c r="D43" s="3">
+        <v>0.34153653976197901</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -2166,11 +2189,11 @@
       <c r="B44">
         <v>2</v>
       </c>
-      <c r="C44">
-        <v>0.55457149663501504</v>
-      </c>
-      <c r="D44">
-        <v>0.24915444372722001</v>
+      <c r="C44" s="3">
+        <v>0.67239861580971905</v>
+      </c>
+      <c r="D44" s="3">
+        <v>0.34087535320762602</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -2180,11 +2203,11 @@
       <c r="B45">
         <v>2</v>
       </c>
-      <c r="C45">
-        <v>0.559968949532613</v>
-      </c>
-      <c r="D45">
-        <v>0.25357209667565</v>
+      <c r="C45" s="3">
+        <v>0.66937120234176595</v>
+      </c>
+      <c r="D45" s="3">
+        <v>0.34214850574343098</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -2194,11 +2217,11 @@
       <c r="B46">
         <v>2</v>
       </c>
-      <c r="C46">
-        <v>0.544523499996591</v>
-      </c>
-      <c r="D46">
-        <v>0.25245876770270198</v>
+      <c r="C46" s="3">
+        <v>0.67083659070713297</v>
+      </c>
+      <c r="D46" s="3">
+        <v>0.34092444184392201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update dependencies and enhance generated figures.
</commit_message>
<xml_diff>
--- a/notebooks/Multi-View Model Performance.xlsx
+++ b/notebooks/Multi-View Model Performance.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29101"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uflorida-my.sharepoint.com/personal/cli2_ufl_edu/Documents/Students/DanielPetti/Projects/SSL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1B969B0-5D00-43E5-9700-BA271903AEF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BF69E1B-E3D6-4917-8CC0-2F8168D1D6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MoCo 2-View" sheetId="1" r:id="rId1"/>
-    <sheet name="MoCo 2-View Synthetic" sheetId="4" r:id="rId2"/>
-    <sheet name="MoCo" sheetId="3" r:id="rId3"/>
-    <sheet name="SimCLR" sheetId="2" r:id="rId4"/>
+    <sheet name="MoCo Temporal" sheetId="5" r:id="rId2"/>
+    <sheet name="MoCo 2-View Synthetic" sheetId="4" r:id="rId3"/>
+    <sheet name="MoCo" sheetId="3" r:id="rId4"/>
+    <sheet name="SimCLR" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="20">
   <si>
     <t>View 1</t>
   </si>
@@ -60,6 +61,9 @@
   </si>
   <si>
     <t>dZ</t>
+  </si>
+  <si>
+    <t>Temporal Gap</t>
   </si>
   <si>
     <t>Model</t>
@@ -154,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -168,6 +172,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1573,6 +1578,197 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6F0B1F5-21C0-47D1-BA4E-DE536194520A}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.5703125" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2">
+        <v>0.5</v>
+      </c>
+      <c r="B2">
+        <v>0.66252612263367605</v>
+      </c>
+      <c r="C2">
+        <v>0.32853140656582003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3">
+        <v>0.5</v>
+      </c>
+      <c r="B3">
+        <v>0.66670617809764898</v>
+      </c>
+      <c r="C3">
+        <v>0.32926154949352598</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>0.5</v>
+      </c>
+      <c r="B4">
+        <v>0.67069955156896599</v>
+      </c>
+      <c r="C4">
+        <v>0.32921990696316</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5">
+        <v>0.1</v>
+      </c>
+      <c r="B5">
+        <v>0.58249987302595196</v>
+      </c>
+      <c r="C5">
+        <v>0.26423979015896998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>0.1</v>
+      </c>
+      <c r="B6">
+        <v>0.58584887285114196</v>
+      </c>
+      <c r="C6">
+        <v>0.26456386437789298</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>0.1</v>
+      </c>
+      <c r="B7">
+        <v>0.58656134941017202</v>
+      </c>
+      <c r="C7">
+        <v>0.26583209620175602</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>0.66812970418564699</v>
+      </c>
+      <c r="C8">
+        <v>0.316088597042537</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>0.68193233844226697</v>
+      </c>
+      <c r="C9">
+        <v>0.32820041914179299</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>0.68835096845514299</v>
+      </c>
+      <c r="C10">
+        <v>0.32990937265771197</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>0</v>
+      </c>
+      <c r="B11">
+        <v>0.70999119143159695</v>
+      </c>
+      <c r="C11">
+        <v>0.35310113623885903</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12">
+        <v>0</v>
+      </c>
+      <c r="B12">
+        <v>0.69610837948953996</v>
+      </c>
+      <c r="C12">
+        <v>0.34927379554863802</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <v>0.70696573983264299</v>
+      </c>
+      <c r="C13">
+        <v>0.359840239692929</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14">
+        <v>1.5</v>
+      </c>
+      <c r="B14">
+        <v>0.63310137654660603</v>
+      </c>
+      <c r="C14">
+        <v>0.28431149153956298</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15">
+        <v>1.5</v>
+      </c>
+      <c r="B15">
+        <v>0.62074537093117899</v>
+      </c>
+      <c r="C15">
+        <v>0.27932704743737002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16">
+        <v>1.5</v>
+      </c>
+      <c r="B16" s="7">
+        <v>0.63531146730453103</v>
+      </c>
+      <c r="C16">
+        <v>0.28609609151549997</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FAB38AB-16FA-4B53-BD8E-E688EAADB5EA}">
   <dimension ref="A1:D46"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2229,7 +2425,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25DEEAC7-22B0-4700-A6E0-9B11E621CA34}">
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2241,7 +2437,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>3</v>
@@ -2252,7 +2448,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <v>0.35310113623885903</v>
@@ -2263,7 +2459,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3">
         <v>0.34927379554863802</v>
@@ -2274,7 +2470,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>0.359840239692929</v>
@@ -2285,7 +2481,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5">
         <v>0.22849317121207799</v>
@@ -2296,7 +2492,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6">
         <v>0.23697700690666601</v>
@@ -2307,7 +2503,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7">
         <v>0.26066549746730999</v>
@@ -2318,7 +2514,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8">
         <v>0.39958888840012302</v>
@@ -2329,7 +2525,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>0.39504857257901099</v>
@@ -2340,7 +2536,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10">
         <v>0.39663225454824902</v>
@@ -2351,7 +2547,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B11">
         <v>0.43066045099536399</v>
@@ -2362,7 +2558,7 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12">
         <v>0.42436723512313901</v>
@@ -2373,7 +2569,7 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>0.42479008271441998</v>
@@ -2384,7 +2580,7 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>0.43648958373278801</v>
@@ -2395,7 +2591,7 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>0.43573921218596501</v>
@@ -2406,7 +2602,7 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16">
         <v>0.43446514722597401</v>
@@ -2417,7 +2613,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B17">
         <v>0.40137972048815002</v>
@@ -2428,7 +2624,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B18">
         <v>0.40141217331836299</v>
@@ -2439,7 +2635,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B19">
         <v>0.39991588894992502</v>
@@ -2450,7 +2646,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B20">
         <v>0.36572818669250301</v>
@@ -2461,7 +2657,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B21">
         <v>0.36838617398301299</v>
@@ -2472,7 +2668,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B22">
         <v>0.36268266964470602</v>
@@ -2483,7 +2679,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B23">
         <v>0.36176116434198902</v>
@@ -2494,7 +2690,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B24">
         <v>0.36137653263139502</v>
@@ -2505,7 +2701,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B25">
         <v>0.36448335108833702</v>
@@ -2516,7 +2712,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B26">
         <v>0.37898444170886397</v>
@@ -2527,7 +2723,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B27">
         <v>0.379589302054893</v>
@@ -2538,7 +2734,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B28">
         <v>0.37687824847312401</v>
@@ -2549,7 +2745,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B29">
         <v>0.37984995987991499</v>
@@ -2560,7 +2756,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B30">
         <v>0.38091644334911501</v>
@@ -2571,7 +2767,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B31">
         <v>0.38014979508164598</v>
@@ -2585,7 +2781,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8489B934-C38F-4048-B81E-B2488082197D}">
   <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2595,7 +2791,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -2606,7 +2802,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <v>0.73952763266819899</v>
@@ -2617,7 +2813,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3">
         <v>0.73413563301777796</v>
@@ -2628,7 +2824,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>0.74359069718377002</v>
@@ -2639,7 +2835,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>0.768245495391913</v>
@@ -2650,7 +2846,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <v>0.76920690472678699</v>
@@ -2661,7 +2857,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7">
         <v>0.77925741809809201</v>
@@ -2672,7 +2868,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8">
         <v>0.78907226047478796</v>
@@ -2683,7 +2879,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>0.78665633934052803</v>
@@ -2694,7 +2890,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10">
         <v>0.78864171836046304</v>
@@ -2705,7 +2901,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11">
         <v>0.80260805806312996</v>
@@ -2716,7 +2912,7 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12">
         <v>0.80089928255171805</v>
@@ -2727,7 +2923,7 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B13">
         <v>0.801113551021715</v>
@@ -2738,7 +2934,7 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B14">
         <v>0.78522753329495598</v>
@@ -2749,7 +2945,7 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B15">
         <v>0.78309162727110904</v>
@@ -2760,7 +2956,7 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16">
         <v>0.78955799945949701</v>
@@ -2771,7 +2967,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B17">
         <v>0.77769010868908095</v>
@@ -2782,7 +2978,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18">
         <v>0.77736646063747605</v>
@@ -2793,7 +2989,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B19">
         <v>0.77588478822501405</v>

</xml_diff>